<commit_message>
Atualiza dados - 18/08/2026 11:10
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F991E8F-2030-400E-9719-FEFA4C61F94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F47D5C3-2113-4E9C-9FA3-FE04BF9231FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="69">
   <si>
     <t>CPF</t>
   </si>
@@ -660,7 +660,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1448,33 +1448,37 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="A8" s="21">
         <v>3596776490</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1" t="s">
-        <v>8</v>
+      <c r="B8" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="22"/>
+      <c r="D8" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
+      <c r="A9" s="21">
         <v>4234381667</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1" t="s">
-        <v>8</v>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="23"/>
+      <c r="E9" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1496,51 +1500,57 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
+      <c r="A11" s="21">
         <v>9293815990</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="4" t="s">
+      <c r="B11" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1" t="s">
-        <v>8</v>
+      <c r="E11" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
+      <c r="A12" s="21">
         <v>14810271153</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="4" t="s">
+      <c r="B12" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1" t="s">
-        <v>8</v>
+      <c r="E12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
+      <c r="A13" s="21">
         <v>34866868368</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1" t="s">
-        <v>8</v>
+      <c r="B13" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1654,17 +1664,19 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
+      <c r="A21" s="21">
         <v>4024368818</v>
       </c>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1" t="s">
-        <v>8</v>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="23"/>
+      <c r="E21" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1682,19 +1694,21 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2">
+      <c r="A23" s="21">
         <v>5863603526</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="4" t="s">
+      <c r="B23" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1" t="s">
-        <v>8</v>
+      <c r="E23" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1912,19 +1926,21 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="2">
+      <c r="A37" s="21">
         <v>3710335</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" s="1"/>
-      <c r="D37" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1" t="s">
-        <v>8</v>
+      <c r="B37" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="22"/>
+      <c r="D37" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -5683,7 +5699,7 @@
   <cols>
     <col min="1" max="1" width="17.44140625" style="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.109375" style="19" customWidth="1"/>
-    <col min="3" max="3" width="211.21875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="140" style="19" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" style="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5716,17 +5732,17 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="27">
+      <c r="A3" s="24">
         <v>2</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="27" t="s">
-        <v>40</v>
+      <c r="D3" s="24" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -5744,17 +5760,17 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="17">
+      <c r="A5" s="27">
         <v>4</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>39</v>
+      <c r="D5" s="27" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -6135,10 +6151,10 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B2" s="13">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C2" s="14">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D2" s="14">
         <v>0</v>
@@ -6151,17 +6167,32 @@
       </c>
       <c r="G2" s="15">
         <f>C2+D2+E2+F2</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="12">
+        <v>11</v>
+      </c>
+      <c r="B3" s="13">
+        <v>46252</v>
+      </c>
+      <c r="C3" s="14">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="15"/>
+      <c r="D3" s="14">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14">
+        <v>0</v>
+      </c>
+      <c r="F3" s="14">
+        <v>2</v>
+      </c>
+      <c r="G3" s="15">
+        <f t="shared" ref="G3:G5" si="0">C3+D3+E3+F3</f>
+        <v>27</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12"/>
@@ -6170,7 +6201,10 @@
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="14"/>
-      <c r="G4" s="15"/>
+      <c r="G4" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12"/>
@@ -6179,7 +6213,10 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
-      <c r="G5" s="15"/>
+      <c r="G5" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza dados - 18/08/2026 11:44
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F47D5C3-2113-4E9C-9FA3-FE04BF9231FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB6E577-CCE0-4200-A7C4-91F14BC81474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="69">
   <si>
     <t>CPF</t>
   </si>
@@ -660,7 +660,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1554,19 +1554,21 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="A14" s="21">
         <v>61902037367</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1" t="s">
-        <v>8</v>
+      <c r="B14" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1858,19 +1860,21 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
+      <c r="A33" s="21">
         <v>68136811091</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="4"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1" t="s">
-        <v>8</v>
+      <c r="B33" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="23"/>
+      <c r="E33" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1944,19 +1948,21 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="2">
+      <c r="A38" s="21">
         <v>6787240</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="1"/>
-      <c r="D38" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1" t="s">
-        <v>8</v>
+      <c r="B38" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="22"/>
+      <c r="D38" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -2118,17 +2124,19 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="2">
+      <c r="A49" s="21">
         <v>9427660</v>
       </c>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="4"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1" t="s">
-        <v>8</v>
+      <c r="B49" s="22"/>
+      <c r="C49" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="23"/>
+      <c r="E49" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F49" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -5731,7 +5739,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="24">
         <v>2</v>
       </c>
@@ -5745,18 +5753,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="27">
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="24">
         <v>3</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="27" t="s">
-        <v>40</v>
+      <c r="D4" s="24" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -5773,7 +5781,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -5787,32 +5795,32 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="17">
-        <v>6</v>
-      </c>
-      <c r="B7" s="18" t="s">
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="27">
+        <v>6</v>
+      </c>
+      <c r="B7" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="17" t="s">
-        <v>39</v>
+      <c r="D7" s="27" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="17">
+      <c r="A8" s="27">
         <v>7</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="17" t="s">
-        <v>39</v>
+      <c r="D8" s="27" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
@@ -5829,7 +5837,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="17">
         <v>9</v>
       </c>
@@ -5843,7 +5851,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A11" s="17">
         <v>10</v>
       </c>
@@ -5871,7 +5879,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="17">
         <v>12</v>
       </c>
@@ -5885,7 +5893,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="17">
         <v>13</v>
       </c>
@@ -5925,7 +5933,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="17">
         <v>16</v>
       </c>
@@ -5939,7 +5947,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="17">
         <v>17</v>
       </c>
@@ -5967,7 +5975,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="17">
         <v>18</v>
       </c>
@@ -5981,7 +5989,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="17">
         <v>20</v>
       </c>
@@ -5995,7 +6003,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="17">
         <v>21</v>
       </c>
@@ -6178,10 +6186,10 @@
         <v>46252</v>
       </c>
       <c r="C3" s="14">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="14">
         <v>0</v>

</xml_diff>

<commit_message>
Atualiza dados - 18/08/2026 11:46
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB6E577-CCE0-4200-A7C4-91F14BC81474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D000EB9-43AF-4D34-99BB-E5B34C72F241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -6186,7 +6186,7 @@
         <v>46252</v>
       </c>
       <c r="C3" s="14">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="14">
         <v>3</v>
@@ -6195,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" s="15">
         <f t="shared" ref="G3:G5" si="0">C3+D3+E3+F3</f>

</xml_diff>

<commit_message>
Atualiza dados - 18/08/2026 11:48
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D000EB9-43AF-4D34-99BB-E5B34C72F241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502A9BB2-EB40-4197-9B4D-11E8289F9789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -5782,17 +5782,17 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="17">
+      <c r="A6" s="27">
         <v>5</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>39</v>
+      <c r="D6" s="27" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza dados - 18/08/2026 15:36
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502A9BB2-EB40-4197-9B4D-11E8289F9789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E81170-E74C-44B9-981E-B1070E843110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="70">
   <si>
     <t>CPF</t>
   </si>
@@ -294,6 +294,9 @@
 Catálogo: Exige autodeclaração = ATIVADO
 Parâmetro:  144 - Fluxo ATESTMED = LIGADO</t>
     </r>
+  </si>
+  <si>
+    <t>Quantidade de Homologadores</t>
   </si>
 </sst>
 </file>
@@ -454,7 +457,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -664,8 +667,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -836,6 +845,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -881,7 +901,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -948,6 +968,20 @@
     <xf numFmtId="0" fontId="0" fillId="37" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1346,19 +1380,21 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="21">
         <v>99418274353</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="22"/>
+      <c r="D2" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
-        <v>8</v>
+      <c r="E2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1572,81 +1608,91 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
+      <c r="A15" s="21">
         <v>73620963649</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1" t="s">
-        <v>8</v>
+      <c r="E15" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
+      <c r="A16" s="21">
         <v>94332096991</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="4" t="s">
+      <c r="B16" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1" t="s">
-        <v>8</v>
+      <c r="E16" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
+      <c r="A17" s="21">
         <v>99894300391</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="4" t="s">
+      <c r="B17" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="22"/>
+      <c r="D17" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1" t="s">
-        <v>8</v>
+      <c r="E17" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="A18" s="21">
         <v>737185309</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="4" t="s">
+      <c r="B18" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1" t="s">
+      <c r="E18" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="22" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
+      <c r="A19" s="21">
         <v>1304390373</v>
       </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1" t="s">
-        <v>8</v>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1682,17 +1728,19 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
+      <c r="A22" s="21">
         <v>5136194960</v>
       </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1" t="s">
-        <v>8</v>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -5702,16 +5750,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.109375" style="19" customWidth="1"/>
-    <col min="3" max="3" width="140" style="19" customWidth="1"/>
+    <col min="3" max="3" width="81.77734375" style="19" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>25</v>
       </c>
@@ -5724,8 +5773,11 @@
       <c r="D1" s="7" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E1" s="30" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="24">
         <v>1</v>
       </c>
@@ -5738,8 +5790,11 @@
       <c r="D2" s="24" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E2" s="35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="24">
         <v>2</v>
       </c>
@@ -5752,8 +5807,11 @@
       <c r="D3" s="24" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E3" s="35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="24">
         <v>3</v>
       </c>
@@ -5766,8 +5824,11 @@
       <c r="D4" s="24" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="27">
         <v>4</v>
       </c>
@@ -5780,8 +5841,11 @@
       <c r="D5" s="27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E5" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="27">
         <v>5</v>
       </c>
@@ -5794,8 +5858,11 @@
       <c r="D6" s="27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E6" s="34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="27">
         <v>6</v>
       </c>
@@ -5808,8 +5875,11 @@
       <c r="D7" s="27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E7" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="27">
         <v>7</v>
       </c>
@@ -5822,64 +5892,79 @@
       <c r="D8" s="27" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="17">
-        <v>8</v>
-      </c>
-      <c r="B9" s="18" t="s">
+      <c r="E8" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="31">
+        <v>8</v>
+      </c>
+      <c r="B9" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="17">
+      <c r="D9" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="31">
         <v>9</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+      <c r="D10" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="31">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+      <c r="D11" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="31">
         <v>11</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D12" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="17">
         <v>12</v>
       </c>
@@ -5892,8 +5977,9 @@
       <c r="D13" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="17">
         <v>13</v>
       </c>
@@ -5906,8 +5992,9 @@
       <c r="D14" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="17">
         <v>14</v>
       </c>
@@ -5918,78 +6005,94 @@
         <v>30</v>
       </c>
       <c r="D15" s="17"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="17">
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="31">
         <v>15</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="17">
+      <c r="D16" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="31">
         <v>16</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="17">
+      <c r="D17" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="31">
         <v>17</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="17">
+      <c r="D18" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="31">
         <v>18</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="17">
+      <c r="D19" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="31">
         <v>18</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D20" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="17">
         <v>20</v>
       </c>
@@ -6002,36 +6105,43 @@
       <c r="D21" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="17">
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="31">
         <v>21</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="17">
+      <c r="D22" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="31">
         <v>22</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D23" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="17">
         <v>23</v>
       </c>
@@ -6044,8 +6154,9 @@
       <c r="D24" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E24" s="9"/>
+    </row>
+    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="17">
         <v>24</v>
       </c>
@@ -6058,22 +6169,26 @@
       <c r="D25" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A26" s="17">
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A26" s="31">
         <v>25</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="D26" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="17">
         <v>26</v>
       </c>
@@ -6086,8 +6201,9 @@
       <c r="D27" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="E27" s="9"/>
+    </row>
+    <row r="28" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A28" s="17">
         <v>27</v>
       </c>
@@ -6100,6 +6216,7 @@
       <c r="D28" s="17" t="s">
         <v>39</v>
       </c>
+      <c r="E28" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza dados - 18/08/2026 16:46
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E81170-E74C-44B9-981E-B1070E843110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAF28B1-D7E6-48D0-99EA-4793879944CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="CENARIOS" sheetId="5" r:id="rId3"/>
     <sheet name="ResumoDiario" sheetId="6" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">CENARIOS!$D$1:$D$28</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="70">
   <si>
     <t>CPF</t>
   </si>
@@ -1696,19 +1699,21 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
+      <c r="A20" s="21">
         <v>2185404938</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="4" t="s">
+      <c r="B20" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1" t="s">
-        <v>8</v>
+      <c r="E20" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1762,51 +1767,57 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
+      <c r="A24" s="21">
         <v>12401303685</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="4" t="s">
+      <c r="B24" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1" t="s">
-        <v>8</v>
+      <c r="E24" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
+      <c r="A25" s="21">
         <v>44771380597</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="4" t="s">
+      <c r="B25" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="22"/>
+      <c r="D25" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1" t="s">
-        <v>8</v>
+      <c r="E25" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
+      <c r="A26" s="21">
         <v>3179868996</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="B26" s="22"/>
+      <c r="C26" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1" t="s">
-        <v>8</v>
+      <c r="E26" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -5210,16 +5221,18 @@
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A243" s="2">
+      <c r="A243" s="21">
         <v>1104046377</v>
       </c>
-      <c r="B243" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C243" s="1"/>
-      <c r="D243" s="4"/>
-      <c r="E243" s="1"/>
-      <c r="F243" s="1" t="s">
+      <c r="B243" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C243" s="22"/>
+      <c r="D243" s="23"/>
+      <c r="E243" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F243" s="22" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5314,17 +5327,19 @@
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A250" s="2">
+      <c r="A250" s="21">
         <v>1327218305</v>
       </c>
-      <c r="B250" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C250" s="1"/>
-      <c r="D250" s="4"/>
-      <c r="E250" s="1"/>
-      <c r="F250" s="1" t="s">
-        <v>8</v>
+      <c r="B250" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C250" s="22"/>
+      <c r="D250" s="23"/>
+      <c r="E250" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F250" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.3">
@@ -5342,33 +5357,37 @@
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A252" s="2">
+      <c r="A252" s="21">
         <v>1520317905</v>
       </c>
-      <c r="B252" s="1"/>
-      <c r="C252" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D252" s="4" t="s">
+      <c r="B252" s="22"/>
+      <c r="C252" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D252" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="E252" s="1"/>
-      <c r="F252" s="1" t="s">
-        <v>8</v>
+      <c r="E252" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F252" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A253" s="2">
+      <c r="A253" s="21">
         <v>1552683257</v>
       </c>
-      <c r="B253" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C253" s="1"/>
-      <c r="D253" s="4"/>
-      <c r="E253" s="1"/>
-      <c r="F253" s="1" t="s">
-        <v>8</v>
+      <c r="B253" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C253" s="22"/>
+      <c r="D253" s="23"/>
+      <c r="E253" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F253" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.3">
@@ -5386,31 +5405,35 @@
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A255" s="2">
+      <c r="A255" s="21">
         <v>1902803280</v>
       </c>
-      <c r="B255" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C255" s="1"/>
-      <c r="D255" s="4"/>
-      <c r="E255" s="1"/>
-      <c r="F255" s="1" t="s">
-        <v>8</v>
+      <c r="B255" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C255" s="22"/>
+      <c r="D255" s="23"/>
+      <c r="E255" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F255" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A256" s="2">
+      <c r="A256" s="21">
         <v>2045280624</v>
       </c>
-      <c r="B256" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C256" s="1"/>
-      <c r="D256" s="4"/>
-      <c r="E256" s="1"/>
-      <c r="F256" s="1" t="s">
-        <v>8</v>
+      <c r="B256" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C256" s="22"/>
+      <c r="D256" s="23"/>
+      <c r="E256" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F256" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.3">
@@ -5430,17 +5453,19 @@
       </c>
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A258" s="2">
+      <c r="A258" s="21">
         <v>2448337292</v>
       </c>
-      <c r="B258" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C258" s="1"/>
-      <c r="D258" s="4"/>
-      <c r="E258" s="1"/>
-      <c r="F258" s="1" t="s">
-        <v>8</v>
+      <c r="B258" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C258" s="22"/>
+      <c r="D258" s="23"/>
+      <c r="E258" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F258" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.3">
@@ -5472,17 +5497,19 @@
       </c>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A261" s="2">
+      <c r="A261" s="21">
         <v>2668682665</v>
       </c>
-      <c r="B261" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C261" s="1"/>
-      <c r="D261" s="4"/>
-      <c r="E261" s="1"/>
-      <c r="F261" s="1" t="s">
-        <v>8</v>
+      <c r="B261" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C261" s="22"/>
+      <c r="D261" s="23"/>
+      <c r="E261" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F261" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.3">
@@ -5530,31 +5557,35 @@
       </c>
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A265" s="2">
+      <c r="A265" s="21">
         <v>3001797150</v>
       </c>
-      <c r="B265" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C265" s="1"/>
-      <c r="D265" s="4"/>
-      <c r="E265" s="1"/>
-      <c r="F265" s="1" t="s">
-        <v>8</v>
+      <c r="B265" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C265" s="22"/>
+      <c r="D265" s="23"/>
+      <c r="E265" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F265" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A266" s="2">
+      <c r="A266" s="21">
         <v>3162488869</v>
       </c>
-      <c r="B266" s="1"/>
-      <c r="C266" s="1"/>
-      <c r="D266" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E266" s="1"/>
-      <c r="F266" s="1" t="s">
-        <v>8</v>
+      <c r="B266" s="22"/>
+      <c r="C266" s="22"/>
+      <c r="D266" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E266" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F266" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -5750,6 +5781,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5777,7 +5809,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="24">
         <v>1</v>
       </c>
@@ -5794,7 +5826,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="24">
         <v>2</v>
       </c>
@@ -5811,7 +5843,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24">
         <v>3</v>
       </c>
@@ -5828,41 +5860,41 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="27">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="24">
         <v>4</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="27">
+      <c r="D5" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="24">
         <v>5</v>
       </c>
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="34">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D6" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="27">
         <v>6</v>
       </c>
@@ -5876,10 +5908,10 @@
         <v>40</v>
       </c>
       <c r="E7" s="34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="27">
         <v>7</v>
       </c>
@@ -5893,10 +5925,10 @@
         <v>40</v>
       </c>
       <c r="E8" s="34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="31">
         <v>8</v>
       </c>
@@ -5913,7 +5945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="31">
         <v>9</v>
       </c>
@@ -5930,7 +5962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="31">
         <v>10</v>
       </c>
@@ -5947,7 +5979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="31">
         <v>11</v>
       </c>
@@ -6004,10 +6036,12 @@
       <c r="C15" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="17"/>
+      <c r="D15" s="17" t="s">
+        <v>39</v>
+      </c>
       <c r="E15" s="9"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="31">
         <v>15</v>
       </c>
@@ -6024,7 +6058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="31">
         <v>16</v>
       </c>
@@ -6041,7 +6075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="31">
         <v>17</v>
       </c>
@@ -6058,7 +6092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="31">
         <v>18</v>
       </c>
@@ -6075,7 +6109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="31">
         <v>18</v>
       </c>
@@ -6107,7 +6141,7 @@
       </c>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="31">
         <v>21</v>
       </c>
@@ -6124,7 +6158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="31">
         <v>22</v>
       </c>
@@ -6171,7 +6205,7 @@
       </c>
       <c r="E25" s="9"/>
     </row>
-    <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="31">
         <v>25</v>
       </c>
@@ -6188,37 +6222,48 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A27" s="17">
+    <row r="27" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="31">
         <v>26</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="D27" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="E27" s="9"/>
-    </row>
-    <row r="28" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A28" s="17">
+      <c r="D27" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="31">
         <v>27</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="E28" s="9"/>
+      <c r="D28" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="E28" s="34">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="D1:D28" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
+    <filterColumn colId="0">
+      <filters blank="1">
+        <filter val="NÃO EXECUTADO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -6303,16 +6348,16 @@
         <v>46252</v>
       </c>
       <c r="C3" s="14">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D3" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E3" s="14">
         <v>0</v>
       </c>
       <c r="F3" s="14">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G3" s="15">
         <f t="shared" ref="G3:G5" si="0">C3+D3+E3+F3</f>

</xml_diff>

<commit_message>
Atualiza dados - 19/08/2026 16:56
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740CBD6E-48FA-47B0-A4A9-9573F5272250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F0C437-60BB-475C-A084-62F2BCE039C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="71">
   <si>
     <t>CPF</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>Possui período validado</t>
+  </si>
+  <si>
+    <t>Ag Reteste</t>
   </si>
 </sst>
 </file>
@@ -460,7 +463,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="41">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -673,6 +676,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -904,7 +919,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -990,6 +1005,26 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2634,39 +2669,43 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="2">
+      <c r="A75" s="18">
         <v>979170796</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D75" s="4" t="s">
+      <c r="B75" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C75" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D75" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1" t="s">
-        <v>7</v>
+      <c r="E75" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F75" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="2">
+      <c r="A76" s="18">
         <v>1017978506</v>
       </c>
-      <c r="B76" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D76" s="4" t="s">
+      <c r="B76" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C76" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1" t="s">
-        <v>7</v>
+      <c r="E76" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F76" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
@@ -2700,19 +2739,21 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="2">
+      <c r="A79" s="18">
         <v>692565</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C79" s="1"/>
-      <c r="D79" s="4" t="s">
+      <c r="B79" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C79" s="19"/>
+      <c r="D79" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1" t="s">
-        <v>7</v>
+      <c r="E79" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F79" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
@@ -5174,17 +5215,19 @@
       </c>
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A237" s="2">
+      <c r="A237" s="18">
         <v>733487246</v>
       </c>
-      <c r="B237" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C237" s="1"/>
-      <c r="D237" s="4"/>
-      <c r="E237" s="1"/>
-      <c r="F237" s="1" t="s">
-        <v>7</v>
+      <c r="B237" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C237" s="19"/>
+      <c r="D237" s="20"/>
+      <c r="E237" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F237" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.3">
@@ -5248,17 +5291,19 @@
       </c>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A242" s="2">
+      <c r="A242" s="18">
         <v>998175277</v>
       </c>
-      <c r="B242" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C242" s="1"/>
-      <c r="D242" s="4"/>
-      <c r="E242" s="1"/>
-      <c r="F242" s="1" t="s">
-        <v>7</v>
+      <c r="B242" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C242" s="19"/>
+      <c r="D242" s="20"/>
+      <c r="E242" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F242" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.3">
@@ -5522,17 +5567,19 @@
       </c>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A260" s="2">
+      <c r="A260" s="18">
         <v>2564074286</v>
       </c>
-      <c r="B260" s="1"/>
-      <c r="C260" s="1"/>
-      <c r="D260" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E260" s="1"/>
-      <c r="F260" s="1" t="s">
-        <v>7</v>
+      <c r="B260" s="19"/>
+      <c r="C260" s="19"/>
+      <c r="D260" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="E260" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F260" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.3">
@@ -5552,33 +5599,37 @@
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A262" s="2">
+      <c r="A262" s="18">
         <v>2705278931</v>
       </c>
-      <c r="B262" s="1"/>
-      <c r="C262" s="1"/>
-      <c r="D262" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E262" s="1"/>
-      <c r="F262" s="1" t="s">
-        <v>7</v>
+      <c r="B262" s="19"/>
+      <c r="C262" s="19"/>
+      <c r="D262" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="E262" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F262" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A263" s="2">
+      <c r="A263" s="18">
         <v>2792829826</v>
       </c>
-      <c r="B263" s="1"/>
-      <c r="C263" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D263" s="4" t="s">
+      <c r="B263" s="19"/>
+      <c r="C263" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D263" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E263" s="1"/>
-      <c r="F263" s="1" t="s">
-        <v>7</v>
+      <c r="E263" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F263" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.3">
@@ -5865,53 +5916,53 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="21">
+      <c r="A3" s="41">
         <v>2</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="29">
+      <c r="D3" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="44">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="33">
+      <c r="A4" s="41">
         <v>3</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="36">
+      <c r="D4" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="44">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="33">
+      <c r="A5" s="41">
         <v>4</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="36">
+      <c r="D5" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="44">
         <v>5</v>
       </c>
     </row>
@@ -6116,7 +6167,7 @@
         <v>39</v>
       </c>
       <c r="E17" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -6133,24 +6184,24 @@
         <v>39</v>
       </c>
       <c r="E18" s="28">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="25">
+      <c r="A19" s="33">
         <v>18</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" s="28">
-        <v>1</v>
+      <c r="D19" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="36">
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -6222,37 +6273,37 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="37">
+      <c r="A24" s="45">
         <v>23</v>
       </c>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="C24" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E24" s="40">
-        <v>0</v>
+      <c r="D24" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" s="48">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="37">
+      <c r="A25" s="45">
         <v>24</v>
       </c>
-      <c r="B25" s="38" t="s">
+      <c r="B25" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="39" t="s">
+      <c r="C25" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E25" s="40">
-        <v>0</v>
+      <c r="D25" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="48">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6326,18 +6377,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABD6A9E0-399C-4737-BBBE-100AAF3BE286}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" customWidth="1"/>
+    <col min="5" max="6" width="15.44140625" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>40</v>
       </c>
@@ -6354,13 +6405,16 @@
         <v>44</v>
       </c>
       <c r="F1" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>0.41666666666666669</v>
       </c>
@@ -6379,12 +6433,15 @@
       <c r="F2" s="14">
         <v>0</v>
       </c>
-      <c r="G2" s="15">
-        <f>C2+D2+E2+F2</f>
+      <c r="G2" s="14">
+        <v>0</v>
+      </c>
+      <c r="H2" s="15">
+        <f>C2+D2+E2+G2+F2</f>
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <v>11</v>
       </c>
@@ -6401,46 +6458,53 @@
         <v>0</v>
       </c>
       <c r="F3" s="14">
+        <v>0</v>
+      </c>
+      <c r="G3" s="14">
         <v>16</v>
       </c>
-      <c r="G3" s="15">
-        <f t="shared" ref="G3:G5" si="0">C3+D3+E3+F3</f>
+      <c r="H3" s="15">
+        <f>C3+D3+E3+G3+F3</f>
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
-        <v>0.64861111111111114</v>
+        <v>0.69791666666666663</v>
       </c>
       <c r="B4" s="13">
         <v>46253</v>
       </c>
       <c r="C4" s="14">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D4" s="14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" s="14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" s="14">
-        <v>6</v>
-      </c>
-      <c r="G4" s="15">
-        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G4" s="14">
+        <v>7</v>
+      </c>
+      <c r="H4" s="15">
+        <f>C4+D4+E4+G4+F4</f>
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12"/>
       <c r="B5" s="13"/>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
-      <c r="G5" s="15">
-        <f t="shared" si="0"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="15">
+        <f t="shared" ref="H3:H5" si="0">C5+D5+E5+G5</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dados - 20/08/2026 11:12
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F0C437-60BB-475C-A084-62F2BCE039C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75585B74-C5A3-460B-A18B-E29A3DD431C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -6239,37 +6239,37 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="37">
+      <c r="A22" s="45">
         <v>21</v>
       </c>
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="39" t="s">
+      <c r="C22" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="40">
-        <v>0</v>
+      <c r="D22" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="48">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="37">
+      <c r="A23" s="45">
         <v>22</v>
       </c>
-      <c r="B23" s="38" t="s">
+      <c r="B23" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="39" t="s">
+      <c r="C23" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" s="40">
-        <v>0</v>
+      <c r="D23" s="45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="48">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -6496,16 +6496,30 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
+      <c r="A5" s="12">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="B5" s="13">
+        <v>46254</v>
+      </c>
+      <c r="C5" s="14">
+        <v>3</v>
+      </c>
+      <c r="D5" s="14">
+        <v>6</v>
+      </c>
+      <c r="E5" s="14">
+        <v>6</v>
+      </c>
+      <c r="F5" s="14">
+        <v>3</v>
+      </c>
+      <c r="G5" s="14">
+        <v>9</v>
+      </c>
       <c r="H5" s="15">
-        <f t="shared" ref="H3:H5" si="0">C5+D5+E5+G5</f>
-        <v>0</v>
+        <f>C5+D5+E5+G5+F5</f>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados - 20/08/2026 12:05
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75585B74-C5A3-460B-A18B-E29A3DD431C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48E165F-6EB5-4B7E-98A5-22369DBE6F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
@@ -6307,20 +6307,20 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="37">
+      <c r="A26" s="33">
         <v>25</v>
       </c>
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E26" s="40">
-        <v>0</v>
+      <c r="D26" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26" s="36">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6503,13 +6503,13 @@
         <v>46254</v>
       </c>
       <c r="C5" s="14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="14">
         <v>6</v>
       </c>
       <c r="E5" s="14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="14">
         <v>3</v>

</xml_diff>

<commit_message>
Atualiza dados - 20/08/2026 16:49
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48E165F-6EB5-4B7E-98A5-22369DBE6F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEA07A8-1763-49A2-88F0-24BB7063A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="71">
   <si>
     <t>CPF</t>
   </si>
@@ -919,7 +919,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -995,16 +995,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1759,19 +1749,17 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="18">
+      <c r="A21" s="30">
         <v>4024368818</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="20"/>
-      <c r="E21" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>5</v>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="32"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2289,19 +2277,21 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="2">
+      <c r="A52" s="18">
         <v>93573006</v>
       </c>
-      <c r="B52" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D52" s="4"/>
-      <c r="E52" s="1"/>
-      <c r="F52" s="1" t="s">
-        <v>7</v>
+      <c r="B52" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" s="20"/>
+      <c r="E52" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F52" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -2453,17 +2443,19 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="2">
+      <c r="A62" s="18">
         <v>2184685550</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C62" s="1"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1" t="s">
-        <v>7</v>
+      <c r="B62" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="19"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -2709,33 +2701,37 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="2">
+      <c r="A77" s="18">
         <v>94893438549</v>
       </c>
-      <c r="B77" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C77" s="1"/>
-      <c r="D77" s="4"/>
-      <c r="E77" s="1"/>
-      <c r="F77" s="1" t="s">
-        <v>7</v>
+      <c r="B77" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="19"/>
+      <c r="D77" s="20"/>
+      <c r="E77" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F77" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="2">
+      <c r="A78" s="18">
         <v>375322</v>
       </c>
-      <c r="B78" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C78" s="1"/>
-      <c r="D78" s="4" t="s">
+      <c r="B78" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="19"/>
+      <c r="D78" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1" t="s">
-        <v>7</v>
+      <c r="E78" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F78" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
@@ -2875,121 +2871,137 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="2">
+      <c r="A87" s="18">
         <v>9229</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C87" s="1"/>
-      <c r="D87" s="4" t="s">
+      <c r="B87" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" s="19"/>
+      <c r="D87" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E87" s="1"/>
-      <c r="F87" s="1" t="s">
-        <v>7</v>
+      <c r="E87" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F87" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="2">
+      <c r="A88" s="18">
         <v>160202</v>
       </c>
-      <c r="B88" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C88" s="1"/>
-      <c r="D88" s="4"/>
-      <c r="E88" s="1"/>
-      <c r="F88" s="1" t="s">
-        <v>7</v>
+      <c r="B88" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" s="19"/>
+      <c r="D88" s="20"/>
+      <c r="E88" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F88" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="2">
+      <c r="A89" s="18">
         <v>176044</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C89" s="1"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="1"/>
-      <c r="F89" s="1" t="s">
-        <v>7</v>
+      <c r="B89" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="19"/>
+      <c r="D89" s="20"/>
+      <c r="E89" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F89" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="2">
+      <c r="A90" s="18">
         <v>352381</v>
       </c>
-      <c r="B90" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C90" s="1"/>
-      <c r="D90" s="4" t="s">
+      <c r="B90" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" s="19"/>
+      <c r="D90" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E90" s="1"/>
-      <c r="F90" s="1" t="s">
-        <v>7</v>
+      <c r="E90" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F90" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="2">
+      <c r="A91" s="18">
         <v>1109570</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C91" s="1"/>
-      <c r="D91" s="4"/>
-      <c r="E91" s="1"/>
-      <c r="F91" s="1" t="s">
-        <v>7</v>
+      <c r="B91" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C91" s="19"/>
+      <c r="D91" s="20"/>
+      <c r="E91" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F91" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="2">
+      <c r="A92" s="18">
         <v>1220330</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C92" s="1"/>
-      <c r="D92" s="4" t="s">
+      <c r="B92" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="19"/>
+      <c r="D92" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E92" s="1"/>
-      <c r="F92" s="1" t="s">
-        <v>7</v>
+      <c r="E92" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F92" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="2">
+      <c r="A93" s="18">
         <v>60129750310</v>
       </c>
-      <c r="B93" s="1"/>
-      <c r="C93" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D93" s="4"/>
-      <c r="E93" s="1"/>
-      <c r="F93" s="1" t="s">
-        <v>7</v>
+      <c r="B93" s="19"/>
+      <c r="C93" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D93" s="20"/>
+      <c r="E93" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F93" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="2">
+      <c r="A94" s="18">
         <v>63707777308</v>
       </c>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D94" s="4"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1" t="s">
-        <v>7</v>
+      <c r="B94" s="19"/>
+      <c r="C94" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D94" s="20"/>
+      <c r="E94" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F94" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
@@ -3165,17 +3177,19 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="2">
+      <c r="A106" s="18">
         <v>6626238</v>
       </c>
-      <c r="B106" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C106" s="1"/>
-      <c r="D106" s="4"/>
-      <c r="E106" s="1"/>
-      <c r="F106" s="1" t="s">
-        <v>7</v>
+      <c r="B106" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C106" s="19"/>
+      <c r="D106" s="20"/>
+      <c r="E106" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F106" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -5319,7 +5333,7 @@
         <v>19</v>
       </c>
       <c r="F243" s="19" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.3">
@@ -5381,19 +5395,21 @@
       </c>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A248" s="2">
+      <c r="A248" s="18">
         <v>1313908215</v>
       </c>
-      <c r="B248" s="1"/>
-      <c r="C248" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D248" s="4" t="s">
+      <c r="B248" s="19"/>
+      <c r="C248" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D248" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E248" s="1"/>
-      <c r="F248" s="1" t="s">
-        <v>7</v>
+      <c r="E248" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F248" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.3">
@@ -5427,17 +5443,19 @@
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A251" s="2">
+      <c r="A251" s="18">
         <v>1469330792</v>
       </c>
-      <c r="B251" s="1"/>
-      <c r="C251" s="1"/>
-      <c r="D251" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E251" s="1"/>
-      <c r="F251" s="1" t="s">
-        <v>7</v>
+      <c r="B251" s="19"/>
+      <c r="C251" s="19"/>
+      <c r="D251" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="E251" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F251" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.3">
@@ -5871,6 +5889,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5898,7 +5917,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21">
         <v>1</v>
       </c>
@@ -5915,58 +5934,58 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="41">
+    <row r="3" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="37">
         <v>2</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="44">
+      <c r="E3" s="40">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="41">
+    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="37">
         <v>3</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="44">
+      <c r="E4" s="40">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="41">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="37">
         <v>4</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="44">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E5" s="40">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>5</v>
       </c>
@@ -5980,75 +5999,75 @@
         <v>35</v>
       </c>
       <c r="E6" s="29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
         <v>6</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="36">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A8" s="33">
-        <v>7</v>
-      </c>
-      <c r="B8" s="34" t="s">
+      <c r="D7" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21">
+        <v>7</v>
+      </c>
+      <c r="B8" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="C8" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="36">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A9" s="33">
+      <c r="D8" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="29">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21">
         <v>8</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="36">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A10" s="25">
+      <c r="D9" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="29">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="37">
         <v>9</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="28">
-        <v>5</v>
+      <c r="D10" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="40">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6065,10 +6084,10 @@
         <v>39</v>
       </c>
       <c r="E11" s="28">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21">
         <v>11</v>
       </c>
@@ -6082,10 +6101,10 @@
         <v>35</v>
       </c>
       <c r="E12" s="29">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="21">
         <v>12</v>
       </c>
@@ -6099,10 +6118,10 @@
         <v>35</v>
       </c>
       <c r="E13" s="29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="21">
         <v>13</v>
       </c>
@@ -6116,10 +6135,10 @@
         <v>35</v>
       </c>
       <c r="E14" s="29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21">
         <v>14</v>
       </c>
@@ -6133,24 +6152,24 @@
         <v>35</v>
       </c>
       <c r="E15" s="29">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="21">
         <v>15</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="28">
-        <v>2</v>
+      <c r="D16" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="29">
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -6170,24 +6189,24 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="25">
+    <row r="18" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="37">
         <v>17</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="28">
+      <c r="D18" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="40">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33">
         <v>18</v>
       </c>
@@ -6205,160 +6224,166 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A20" s="33">
+      <c r="A20" s="25">
         <v>19</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="36">
+      <c r="D20" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="33">
+      <c r="A21" s="25">
         <v>20</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E21" s="36">
+      <c r="D21" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="45">
+      <c r="A22" s="41">
         <v>21</v>
       </c>
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="47" t="s">
+      <c r="C22" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="45" t="s">
+      <c r="D22" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="48">
+      <c r="E22" s="44">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="45">
+      <c r="A23" s="41">
         <v>22</v>
       </c>
-      <c r="B23" s="46" t="s">
+      <c r="B23" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="47" t="s">
+      <c r="C23" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="45" t="s">
+      <c r="D23" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="E23" s="48">
+      <c r="E23" s="44">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="45">
+      <c r="A24" s="41">
         <v>23</v>
       </c>
-      <c r="B24" s="46" t="s">
+      <c r="B24" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="47" t="s">
+      <c r="C24" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="45" t="s">
+      <c r="D24" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="E24" s="48">
+      <c r="E24" s="44">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="45">
+      <c r="A25" s="41">
         <v>24</v>
       </c>
-      <c r="B25" s="46" t="s">
+      <c r="B25" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="47" t="s">
+      <c r="C25" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="45" t="s">
+      <c r="D25" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="48">
+      <c r="E25" s="44">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="33">
+      <c r="A26" s="25">
         <v>25</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B26" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="35" t="s">
+      <c r="C26" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E26" s="36">
+      <c r="D26" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="28">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="37">
+      <c r="A27" s="25">
         <v>26</v>
       </c>
-      <c r="B27" s="38" t="s">
+      <c r="B27" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="39" t="s">
+      <c r="C27" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="40">
-        <v>0</v>
+      <c r="D27" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="28">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="37">
+      <c r="A28" s="25">
         <v>27</v>
       </c>
-      <c r="B28" s="38" t="s">
+      <c r="B28" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E28" s="40">
-        <v>0</v>
+      <c r="D28" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D28" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}"/>
+  <autoFilter ref="D1:D28" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="EM TESTE"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -6497,25 +6522,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
-        <v>0.45833333333333331</v>
+        <v>0.69930555555555551</v>
       </c>
       <c r="B5" s="13">
         <v>46254</v>
       </c>
       <c r="C5" s="14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E5" s="14">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F5" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G5" s="14">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H5" s="15">
         <f>C5+D5+E5+G5+F5</f>

</xml_diff>

<commit_message>
Atualiza dados - 21/08/2026 11:45
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEA07A8-1763-49A2-88F0-24BB7063A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70E7D14-7EC5-4C72-AFE3-0E3C07279779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -20,6 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">CENARIOS!$D$1:$D$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Massa_HML_B31_FLUXO_INTEGRADO!$A$1:$F$266</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="71">
   <si>
     <t>CPF</t>
   </si>
@@ -463,7 +464,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -676,12 +677,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -919,7 +914,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -985,16 +980,6 @@
     <xf numFmtId="164" fontId="0" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1005,16 +990,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1381,6 +1356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834A0C64-4F07-424E-993E-2EA5E6BA9836}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F266"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1461,7 +1437,7 @@
         <v>16</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1711,7 +1687,7 @@
         <v>15</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1748,7 +1724,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="30">
         <v>4024368818</v>
       </c>
@@ -1908,7 +1884,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>17713986987</v>
       </c>
@@ -1924,7 +1900,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>20404965806</v>
       </c>
@@ -2014,7 +1990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>87764997404</v>
       </c>
@@ -2066,7 +2042,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>9366261</v>
       </c>
@@ -2082,7 +2058,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>1548301</v>
       </c>
@@ -2098,7 +2074,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>1818384</v>
       </c>
@@ -2114,7 +2090,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>59054271</v>
       </c>
@@ -2130,7 +2106,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>65913299</v>
       </c>
@@ -2146,7 +2122,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>79277209</v>
       </c>
@@ -2162,7 +2138,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>79682219</v>
       </c>
@@ -2176,7 +2152,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>102850240</v>
       </c>
@@ -2190,7 +2166,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>114745218</v>
       </c>
@@ -2206,7 +2182,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>7227906</v>
       </c>
@@ -2240,7 +2216,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>10152148</v>
       </c>
@@ -2258,7 +2234,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>61461121</v>
       </c>
@@ -2294,7 +2270,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>95026100</v>
       </c>
@@ -2310,7 +2286,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>7494173404</v>
       </c>
@@ -2328,7 +2304,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>7496954390</v>
       </c>
@@ -2346,7 +2322,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>7502772383</v>
       </c>
@@ -2381,22 +2357,24 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="2">
+      <c r="A58" s="18">
         <v>251275</v>
       </c>
-      <c r="B58" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C58" s="1"/>
-      <c r="D58" s="4" t="s">
+      <c r="B58" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="19"/>
+      <c r="D58" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E58" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F58" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>40999408</v>
       </c>
@@ -2412,7 +2390,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>52062511</v>
       </c>
@@ -2426,7 +2404,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>96619309</v>
       </c>
@@ -2458,7 +2436,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>136679390</v>
       </c>
@@ -2476,7 +2454,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>284905330</v>
       </c>
@@ -2492,7 +2470,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>404822606</v>
       </c>
@@ -2510,7 +2488,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>455785163</v>
       </c>
@@ -2528,7 +2506,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>485318989</v>
       </c>
@@ -2544,7 +2522,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>98983768304</v>
       </c>
@@ -2558,7 +2536,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>99052210349</v>
       </c>
@@ -2574,7 +2552,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>99178826500</v>
       </c>
@@ -2588,7 +2566,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>99447444504</v>
       </c>
@@ -2753,22 +2731,24 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="2">
+      <c r="A80" s="18">
         <v>867039</v>
       </c>
-      <c r="B80" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C80" s="1"/>
-      <c r="D80" s="4" t="s">
+      <c r="B80" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C80" s="19"/>
+      <c r="D80" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E80" s="1"/>
-      <c r="F80" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E80" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F80" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>9955937289</v>
       </c>
@@ -2784,7 +2764,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>15930796998</v>
       </c>
@@ -2803,22 +2783,24 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="2">
+      <c r="A83" s="18">
         <v>15930802980</v>
       </c>
-      <c r="B83" s="1"/>
-      <c r="C83" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D83" s="4" t="s">
+      <c r="B83" s="19"/>
+      <c r="C83" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D83" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E83" s="1"/>
-      <c r="F83" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E83" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F83" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>20603332889</v>
       </c>
@@ -2835,39 +2817,43 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="2">
+      <c r="A85" s="18">
         <v>31828499803</v>
       </c>
-      <c r="B85" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D85" s="4" t="s">
+      <c r="B85" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D85" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E85" s="1"/>
-      <c r="F85" s="1" t="s">
-        <v>7</v>
+      <c r="E85" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F85" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="2">
+      <c r="A86" s="18">
         <v>75424460291</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D86" s="4" t="s">
+      <c r="B86" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C86" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D86" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E86" s="1"/>
-      <c r="F86" s="1" t="s">
-        <v>7</v>
+      <c r="E86" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F86" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
@@ -3004,7 +2990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>94410984349</v>
       </c>
@@ -3018,7 +3004,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>1943263302</v>
       </c>
@@ -3034,7 +3020,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>3293140335</v>
       </c>
@@ -3050,7 +3036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>11302822365</v>
       </c>
@@ -3082,7 +3068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>49293710153</v>
       </c>
@@ -3096,7 +3082,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>62206311615</v>
       </c>
@@ -3112,7 +3098,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>1409107</v>
       </c>
@@ -3128,7 +3114,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>1455133</v>
       </c>
@@ -3144,7 +3130,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>1524208</v>
       </c>
@@ -3160,7 +3146,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>5165202</v>
       </c>
@@ -3192,7 +3178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>1754503586</v>
       </c>
@@ -3210,7 +3196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>2820058205</v>
       </c>
@@ -3226,7 +3212,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>4099781674</v>
       </c>
@@ -3243,19 +3229,21 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="2">
+      <c r="A110" s="18">
         <v>5485659101</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C110" s="1"/>
-      <c r="D110" s="4" t="s">
+      <c r="B110" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C110" s="19"/>
+      <c r="D110" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E110" s="1"/>
-      <c r="F110" s="1" t="s">
-        <v>7</v>
+      <c r="E110" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F110" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -3290,7 +3278,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>1872891071</v>
       </c>
@@ -3308,7 +3296,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>6300019446</v>
       </c>
@@ -3322,7 +3310,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>7297222445</v>
       </c>
@@ -3368,7 +3356,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>1827618</v>
       </c>
@@ -3382,7 +3370,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>1834584</v>
       </c>
@@ -3399,20 +3387,22 @@
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="2">
+      <c r="A120" s="18">
         <v>17382940802</v>
       </c>
-      <c r="B120" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C120" s="1"/>
-      <c r="D120" s="4"/>
-      <c r="E120" s="1"/>
-      <c r="F120" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B120" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C120" s="19"/>
+      <c r="D120" s="20"/>
+      <c r="E120" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F120" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>61707357323</v>
       </c>
@@ -3427,22 +3417,24 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="2">
+      <c r="A122" s="18">
         <v>5361133</v>
       </c>
-      <c r="B122" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C122" s="1"/>
-      <c r="D122" s="4" t="s">
+      <c r="B122" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C122" s="19"/>
+      <c r="D122" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E122" s="1"/>
-      <c r="F122" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E122" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F122" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>11194359</v>
       </c>
@@ -3458,7 +3450,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>35324376</v>
       </c>
@@ -3474,7 +3466,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>36184390</v>
       </c>
@@ -3490,7 +3482,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>92359426320</v>
       </c>
@@ -3506,7 +3498,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>2149575</v>
       </c>
@@ -3522,7 +3514,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>3382076519</v>
       </c>
@@ -3538,7 +3530,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>56905580520</v>
       </c>
@@ -3554,7 +3546,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>284471313</v>
       </c>
@@ -3572,7 +3564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>95044353191</v>
       </c>
@@ -3588,7 +3580,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>87026902172</v>
       </c>
@@ -3604,7 +3596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>74802585268</v>
       </c>
@@ -3622,7 +3614,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>64074072149</v>
       </c>
@@ -3638,7 +3630,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>3633872345</v>
       </c>
@@ -3656,7 +3648,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>103076301</v>
       </c>
@@ -3674,7 +3666,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>1167202635</v>
       </c>
@@ -3692,7 +3684,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>56919069504</v>
       </c>
@@ -3710,7 +3702,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>13080839633</v>
       </c>
@@ -3726,7 +3718,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>97485632515</v>
       </c>
@@ -3744,7 +3736,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>11202344410</v>
       </c>
@@ -3760,7 +3752,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>7167052302</v>
       </c>
@@ -3778,7 +3770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>6398143604</v>
       </c>
@@ -3794,7 +3786,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>2331911355</v>
       </c>
@@ -3810,7 +3802,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>16874878638</v>
       </c>
@@ -3826,7 +3818,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>44367066304</v>
       </c>
@@ -3842,7 +3834,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>46272803869</v>
       </c>
@@ -3858,7 +3850,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>32298315191</v>
       </c>
@@ -3874,7 +3866,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>8888285601</v>
       </c>
@@ -3890,7 +3882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>1615275401</v>
       </c>
@@ -3908,7 +3900,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>6011652760</v>
       </c>
@@ -3924,7 +3916,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>57908893104</v>
       </c>
@@ -3942,7 +3934,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>70586931295</v>
       </c>
@@ -3958,7 +3950,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>97407828253</v>
       </c>
@@ -3974,7 +3966,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>3017306607</v>
       </c>
@@ -3990,7 +3982,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>11431230421</v>
       </c>
@@ -4006,7 +3998,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>1705491359</v>
       </c>
@@ -4022,7 +4014,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>92055613553</v>
       </c>
@@ -4040,7 +4032,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>4434895303</v>
       </c>
@@ -4058,7 +4050,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>5724205602</v>
       </c>
@@ -4074,7 +4066,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>3670862048</v>
       </c>
@@ -4092,7 +4084,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>8874532792</v>
       </c>
@@ -4110,7 +4102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>62602713287</v>
       </c>
@@ -4128,7 +4120,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>9006781940</v>
       </c>
@@ -4160,7 +4152,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>11652859918</v>
       </c>
@@ -4176,7 +4168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2">
         <v>14693733601</v>
       </c>
@@ -4192,7 +4184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2">
         <v>93842155620</v>
       </c>
@@ -4208,7 +4200,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>32762364</v>
       </c>
@@ -4224,7 +4216,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>38628015</v>
       </c>
@@ -4240,7 +4232,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>71667377</v>
       </c>
@@ -4254,7 +4246,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>251356</v>
       </c>
@@ -4270,7 +4262,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>995207</v>
       </c>
@@ -4286,7 +4278,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>1322338</v>
       </c>
@@ -4302,7 +4294,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>5211913</v>
       </c>
@@ -4316,7 +4308,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>54783321</v>
       </c>
@@ -4332,7 +4324,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2">
         <v>187948313</v>
       </c>
@@ -4348,7 +4340,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
         <v>1175017</v>
       </c>
@@ -4364,7 +4356,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="2">
         <v>13693778</v>
       </c>
@@ -4378,7 +4370,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="2">
         <v>19595905</v>
       </c>
@@ -4394,7 +4386,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="2">
         <v>72335319</v>
       </c>
@@ -4410,7 +4402,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2">
         <v>141827343</v>
       </c>
@@ -4426,7 +4418,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="2">
         <v>152671307</v>
       </c>
@@ -4440,7 +4432,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="2">
         <v>176295356</v>
       </c>
@@ -4456,7 +4448,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="2">
         <v>188854037</v>
       </c>
@@ -4471,78 +4463,88 @@
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A186" s="2">
+      <c r="A186" s="18">
         <v>261974050</v>
       </c>
-      <c r="B186" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C186" s="1"/>
-      <c r="D186" s="4"/>
-      <c r="E186" s="1"/>
-      <c r="F186" s="1" t="s">
-        <v>7</v>
+      <c r="B186" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C186" s="19"/>
+      <c r="D186" s="20"/>
+      <c r="E186" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F186" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A187" s="2">
+      <c r="A187" s="18">
         <v>279698003</v>
       </c>
-      <c r="B187" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C187" s="1"/>
-      <c r="D187" s="4" t="s">
+      <c r="B187" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C187" s="19"/>
+      <c r="D187" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E187" s="1"/>
-      <c r="F187" s="1" t="s">
-        <v>7</v>
+      <c r="E187" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F187" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A188" s="2">
+      <c r="A188" s="18">
         <v>313186308</v>
       </c>
-      <c r="B188" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C188" s="1"/>
-      <c r="D188" s="4"/>
-      <c r="E188" s="1"/>
-      <c r="F188" s="1" t="s">
-        <v>7</v>
+      <c r="B188" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C188" s="19"/>
+      <c r="D188" s="20"/>
+      <c r="E188" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F188" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A189" s="2">
+      <c r="A189" s="18">
         <v>342804057</v>
       </c>
-      <c r="B189" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C189" s="1"/>
-      <c r="D189" s="4"/>
-      <c r="E189" s="1"/>
-      <c r="F189" s="1" t="s">
-        <v>7</v>
+      <c r="B189" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C189" s="19"/>
+      <c r="D189" s="20"/>
+      <c r="E189" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F189" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A190" s="2">
+      <c r="A190" s="18">
         <v>413071006</v>
       </c>
-      <c r="B190" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C190" s="1"/>
-      <c r="D190" s="4"/>
-      <c r="E190" s="1"/>
-      <c r="F190" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B190" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C190" s="19"/>
+      <c r="D190" s="20"/>
+      <c r="E190" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F190" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="2">
         <v>415141222</v>
       </c>
@@ -4558,7 +4560,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2">
         <v>420585540</v>
       </c>
@@ -4574,7 +4576,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="2">
         <v>90200551</v>
       </c>
@@ -4592,7 +4594,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="2">
         <v>408855509</v>
       </c>
@@ -4610,7 +4612,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="2">
         <v>3867409501</v>
       </c>
@@ -4628,7 +4630,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="2">
         <v>4449548647</v>
       </c>
@@ -4644,7 +4646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="2">
         <v>4723145486</v>
       </c>
@@ -4662,7 +4664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2">
         <v>149071</v>
       </c>
@@ -4676,7 +4678,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="2">
         <v>6272320</v>
       </c>
@@ -4692,7 +4694,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="2">
         <v>6313531</v>
       </c>
@@ -4708,7 +4710,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="2">
         <v>6340342</v>
       </c>
@@ -4722,7 +4724,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="2">
         <v>7231342</v>
       </c>
@@ -4738,7 +4740,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="2">
         <v>11528311</v>
       </c>
@@ -4752,7 +4754,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="2">
         <v>247324</v>
       </c>
@@ -4766,7 +4768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="2">
         <v>308307</v>
       </c>
@@ -4781,20 +4783,22 @@
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A206" s="2">
+      <c r="A206" s="18">
         <v>2822350</v>
       </c>
-      <c r="B206" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C206" s="1"/>
-      <c r="D206" s="4"/>
-      <c r="E206" s="1"/>
-      <c r="F206" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B206" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C206" s="19"/>
+      <c r="D206" s="20"/>
+      <c r="E206" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F206" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="2">
         <v>3469344</v>
       </c>
@@ -4808,7 +4812,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="2">
         <v>4868250</v>
       </c>
@@ -4822,7 +4826,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="2">
         <v>5743095</v>
       </c>
@@ -4836,7 +4840,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="2">
         <v>1450336</v>
       </c>
@@ -4850,7 +4854,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="2">
         <v>1703307</v>
       </c>
@@ -4864,7 +4868,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="2">
         <v>2613352</v>
       </c>
@@ -4880,7 +4884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="2">
         <v>2621533</v>
       </c>
@@ -4894,7 +4898,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="2">
         <v>3708276</v>
       </c>
@@ -4910,7 +4914,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="2">
         <v>8201936582</v>
       </c>
@@ -4924,7 +4928,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="2">
         <v>636304</v>
       </c>
@@ -4940,7 +4944,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="2">
         <v>1694200</v>
       </c>
@@ -4954,7 +4958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="2">
         <v>4889339</v>
       </c>
@@ -4968,7 +4972,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="2">
         <v>5079381</v>
       </c>
@@ -4982,7 +4986,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" s="2">
         <v>5114390</v>
       </c>
@@ -4996,7 +5000,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="2">
         <v>5265339</v>
       </c>
@@ -5010,7 +5014,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="2">
         <v>11964723</v>
       </c>
@@ -5040,7 +5044,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" s="2">
         <v>156788730</v>
       </c>
@@ -5056,7 +5060,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="2">
         <v>221921745</v>
       </c>
@@ -5071,20 +5075,22 @@
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A226" s="2">
+      <c r="A226" s="18">
         <v>247862258</v>
       </c>
-      <c r="B226" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C226" s="1"/>
-      <c r="D226" s="4"/>
-      <c r="E226" s="1"/>
-      <c r="F226" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B226" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C226" s="19"/>
+      <c r="D226" s="20"/>
+      <c r="E226" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F226" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="2">
         <v>260357588</v>
       </c>
@@ -5098,7 +5104,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="2">
         <v>281685770</v>
       </c>
@@ -5112,7 +5118,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="2">
         <v>303117214</v>
       </c>
@@ -5126,7 +5132,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="2">
         <v>345513878</v>
       </c>
@@ -5140,7 +5146,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="2">
         <v>393343766</v>
       </c>
@@ -5155,20 +5161,22 @@
       </c>
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A232" s="2">
+      <c r="A232" s="18">
         <v>404870406</v>
       </c>
-      <c r="B232" s="1"/>
-      <c r="C232" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D232" s="4"/>
-      <c r="E232" s="1"/>
-      <c r="F232" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B232" s="19"/>
+      <c r="C232" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D232" s="20"/>
+      <c r="E232" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F232" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="2">
         <v>415001994</v>
       </c>
@@ -5184,7 +5192,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="2">
         <v>417375638</v>
       </c>
@@ -5200,7 +5208,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="2">
         <v>461926709</v>
       </c>
@@ -5214,7 +5222,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="2">
         <v>505870568</v>
       </c>
@@ -5244,7 +5252,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="2">
         <v>866715029</v>
       </c>
@@ -5258,7 +5266,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="2">
         <v>876775202</v>
       </c>
@@ -5275,33 +5283,37 @@
       </c>
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A240" s="2">
+      <c r="A240" s="18">
         <v>965936953</v>
       </c>
-      <c r="B240" s="1"/>
-      <c r="C240" s="1"/>
-      <c r="D240" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E240" s="1"/>
-      <c r="F240" s="1" t="s">
-        <v>7</v>
+      <c r="B240" s="19"/>
+      <c r="C240" s="19"/>
+      <c r="D240" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="E240" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F240" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A241" s="2">
+      <c r="A241" s="18">
         <v>980772796</v>
       </c>
-      <c r="B241" s="1"/>
-      <c r="C241" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D241" s="4" t="s">
+      <c r="B241" s="19"/>
+      <c r="C241" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D241" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="E241" s="1"/>
-      <c r="F241" s="1" t="s">
-        <v>7</v>
+      <c r="E241" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F241" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.3">
@@ -5336,7 +5348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="2">
         <v>1129136876</v>
       </c>
@@ -5350,7 +5362,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" s="2">
         <v>1215211767</v>
       </c>
@@ -5364,7 +5376,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="2">
         <v>1270440276</v>
       </c>
@@ -5380,7 +5392,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" s="2">
         <v>1309511101</v>
       </c>
@@ -5412,7 +5424,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="2">
         <v>1316735214</v>
       </c>
@@ -5429,17 +5441,19 @@
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A250" s="30">
+      <c r="A250" s="18">
         <v>1327218305</v>
       </c>
-      <c r="B250" s="31" t="s">
-        <v>5</v>
-      </c>
-      <c r="C250" s="31"/>
-      <c r="D250" s="32"/>
-      <c r="E250" s="31"/>
-      <c r="F250" s="31" t="s">
-        <v>7</v>
+      <c r="B250" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C250" s="19"/>
+      <c r="D250" s="20"/>
+      <c r="E250" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F250" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.3">
@@ -5492,7 +5506,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="2">
         <v>1752772733</v>
       </c>
@@ -5538,7 +5552,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="2">
         <v>2346482285</v>
       </c>
@@ -5570,7 +5584,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="2">
         <v>2467922480</v>
       </c>
@@ -5650,7 +5664,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" s="2">
         <v>2936656729</v>
       </c>
@@ -5697,6 +5711,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F266" xr:uid="{834A0C64-4F07-424E-993E-2EA5E6BA9836}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="SIM"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="A2:F2">
     <cfRule type="cellIs" dxfId="0" priority="2" stopIfTrue="1" operator="greaterThan">
       <formula>$F$2="SIM"</formula>
@@ -5935,53 +5956,53 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37">
+      <c r="A3" s="21">
         <v>2</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="40">
-        <v>6</v>
+      <c r="D3" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="29">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="37">
+      <c r="A4" s="21">
         <v>3</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="40">
-        <v>6</v>
+      <c r="D4" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="29">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37">
+      <c r="A5" s="21">
         <v>4</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E5" s="40">
+      <c r="D5" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="29">
         <v>6</v>
       </c>
     </row>
@@ -6054,20 +6075,20 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="21">
         <v>9</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="40">
-        <v>7</v>
+      <c r="D10" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="29">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6172,54 +6193,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="25">
+    <row r="17" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="21">
         <v>16</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="28">
-        <v>2</v>
+      <c r="D17" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="29">
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="37">
+      <c r="A18" s="21">
         <v>17</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="40">
+      <c r="D18" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="29">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33">
+      <c r="A19" s="21">
         <v>18</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="36">
+      <c r="D19" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="29">
         <v>3</v>
       </c>
     </row>
@@ -6237,92 +6258,92 @@
         <v>39</v>
       </c>
       <c r="E20" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="21">
         <v>20</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="27" t="s">
+      <c r="C21" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="21">
+        <v>21</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="33">
+        <v>22</v>
+      </c>
+      <c r="B23" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E21" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="41">
-        <v>21</v>
-      </c>
-      <c r="B22" s="42" t="s">
+      <c r="E23" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="33">
+        <v>23</v>
+      </c>
+      <c r="B24" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="41" t="s">
+      <c r="C24" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="41">
-        <v>22</v>
-      </c>
-      <c r="B23" s="42" t="s">
+      <c r="E24" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="33">
+        <v>24</v>
+      </c>
+      <c r="B25" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="43" t="s">
-        <v>29</v>
-      </c>
-      <c r="D23" s="41" t="s">
+      <c r="C25" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E23" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="41">
-        <v>23</v>
-      </c>
-      <c r="B24" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="43" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="41">
-        <v>24</v>
-      </c>
-      <c r="B25" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="D25" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="E25" s="44">
-        <v>1</v>
+      <c r="E25" s="36">
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6356,7 +6377,7 @@
         <v>39</v>
       </c>
       <c r="E27" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6373,7 +6394,7 @@
         <v>39</v>
       </c>
       <c r="E28" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -6522,7 +6543,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
-        <v>0.69930555555555551</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="B5" s="13">
         <v>46254</v>
@@ -6531,16 +6552,16 @@
         <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E5" s="14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G5" s="14">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H5" s="15">
         <f>C5+D5+E5+G5+F5</f>

</xml_diff>

<commit_message>
Atualiza dados - 21/08/2026 11:58
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70E7D14-7EC5-4C72-AFE3-0E3C07279779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BBF23C-483B-423F-822B-127EBFE39001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -6296,20 +6296,20 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="33">
+      <c r="A23" s="21">
         <v>22</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E23" s="36">
-        <v>2</v>
+      <c r="D23" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="29">
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -6360,7 +6360,7 @@
         <v>39</v>
       </c>
       <c r="E26" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6552,7 +6552,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" s="14">
         <v>0</v>
@@ -6561,7 +6561,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H5" s="15">
         <f>C5+D5+E5+G5+F5</f>

</xml_diff>

<commit_message>
Atualiza dados - 21/08/2026 15:10
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BBF23C-483B-423F-822B-127EBFE39001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5238F3-D575-4B89-BC64-AE9CF42D76A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -6245,20 +6245,20 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A20" s="25">
+      <c r="A20" s="21">
         <v>19</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="28">
-        <v>2</v>
+      <c r="D20" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="29">
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
@@ -6295,7 +6295,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="21">
         <v>22</v>
       </c>
@@ -6312,20 +6312,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="33">
+    <row r="24" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="21">
         <v>23</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="36">
+      <c r="D24" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="29">
         <v>2</v>
       </c>
     </row>
@@ -6346,55 +6346,55 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="25">
+    <row r="26" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="21">
         <v>25</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E26" s="28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="25">
+      <c r="D26" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="21">
         <v>26</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E27" s="28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="25">
+      <c r="D27" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" s="29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="21">
         <v>27</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E28" s="28">
-        <v>2</v>
+      <c r="D28" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="29">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -6552,7 +6552,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="14">
         <v>0</v>
@@ -6561,7 +6561,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H5" s="15">
         <f>C5+D5+E5+G5+F5</f>

</xml_diff>

<commit_message>
Atualiza dados - 21/08/2026 15:12
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5238F3-D575-4B89-BC64-AE9CF42D76A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B605C3-3F61-49EF-B6F2-968E4C751D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -5910,7 +5910,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5938,7 +5937,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="21">
         <v>1</v>
       </c>
@@ -5955,7 +5954,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>2</v>
       </c>
@@ -5972,7 +5971,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="21">
         <v>3</v>
       </c>
@@ -5989,7 +5988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="21">
         <v>4</v>
       </c>
@@ -6006,7 +6005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>5</v>
       </c>
@@ -6023,7 +6022,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>6</v>
       </c>
@@ -6040,7 +6039,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>7</v>
       </c>
@@ -6057,7 +6056,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A9" s="21">
         <v>8</v>
       </c>
@@ -6074,7 +6073,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="21">
         <v>9</v>
       </c>
@@ -6108,7 +6107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="21">
         <v>11</v>
       </c>
@@ -6125,7 +6124,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="21">
         <v>12</v>
       </c>
@@ -6142,7 +6141,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="21">
         <v>13</v>
       </c>
@@ -6159,7 +6158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="21">
         <v>14</v>
       </c>
@@ -6176,7 +6175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="21">
         <v>15</v>
       </c>
@@ -6193,7 +6192,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="21">
         <v>16</v>
       </c>
@@ -6210,7 +6209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="21">
         <v>17</v>
       </c>
@@ -6227,7 +6226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A19" s="21">
         <v>18</v>
       </c>
@@ -6261,7 +6260,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A21" s="21">
         <v>20</v>
       </c>
@@ -6278,7 +6277,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A22" s="21">
         <v>21</v>
       </c>
@@ -6295,7 +6294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="21">
         <v>22</v>
       </c>
@@ -6312,7 +6311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="21">
         <v>23</v>
       </c>
@@ -6346,7 +6345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A26" s="21">
         <v>25</v>
       </c>
@@ -6363,7 +6362,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A27" s="21">
         <v>26</v>
       </c>
@@ -6380,7 +6379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="21">
         <v>27</v>
       </c>
@@ -6398,13 +6397,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D28" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="EM TESTE"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="D1:D28" xr:uid="{9A07569E-5BDC-415E-ABD1-103C61B67D37}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -6543,25 +6536,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
-        <v>0.47916666666666669</v>
+        <v>0.625</v>
       </c>
       <c r="B5" s="13">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C5" s="14">
         <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E5" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="14">
         <v>0</v>
       </c>
       <c r="G5" s="14">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H5" s="15">
         <f>C5+D5+E5+G5+F5</f>

</xml_diff>

<commit_message>
Atualiza dados - 21/08/2026 16:48
</commit_message>
<xml_diff>
--- a/fluxo-integrado/Massa_CPFs_FPSE.xlsx
+++ b/fluxo-integrado/Massa_CPFs_FPSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fluxo-integrado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B605C3-3F61-49EF-B6F2-968E4C751D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F04A8A-9EA2-47BE-9448-392D31835AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{59B77761-AE3C-4E52-A7E7-6436E081B1B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Massa_HML_B31_FLUXO_INTEGRADO" sheetId="3" r:id="rId1"/>
@@ -464,7 +464,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -677,12 +677,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -914,7 +908,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -980,16 +974,6 @@
     <xf numFmtId="164" fontId="0" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -6325,24 +6309,24 @@
         <v>35</v>
       </c>
       <c r="E24" s="29">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="33">
+      <c r="A25" s="21">
         <v>24</v>
       </c>
-      <c r="B25" s="34" t="s">
+      <c r="B25" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="E25" s="36">
-        <v>2</v>
+      <c r="D25" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" s="29">
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
@@ -6545,10 +6529,10 @@
         <v>0</v>
       </c>
       <c r="D5" s="14">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="14">
         <v>0</v>

</xml_diff>